<commit_message>
paper run 2026-10-14 09:42
</commit_message>
<xml_diff>
--- a/reports/2026-10-14.xlsx
+++ b/reports/2026-10-14.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -681,13 +681,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>-149.25</v>
+        <v>-70.34</v>
       </c>
       <c r="E15" t="n">
         <v>-4.64</v>
@@ -707,13 +707,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>-149.25</v>
+        <v>-70.34</v>
       </c>
       <c r="E17" t="n">
         <v>-4.64</v>
@@ -748,261 +748,299 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>78.91</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>-149.25</v>
-      </c>
-      <c r="E21" t="n">
-        <v>-4.64</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>78.91</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-149.25</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-4.64</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" t="n">
-        <v>-4.64</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-4.64</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="n">
-        <v>-4.64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-4.64</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" t="n">
-        <v>-4.64</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-4.64</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
-        <v>-4.64</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-4.64</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="n">
-        <v>-4.64</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-4.64</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" t="n">
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
         <v>-4.64</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-10-14 17:00
</commit_message>
<xml_diff>
--- a/reports/2026-10-14.xlsx
+++ b/reports/2026-10-14.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,92 @@
       </c>
       <c r="K2" t="n">
         <v>-4.64</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-14T14:23:57.235382+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F3" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="G3" t="n">
+        <v>13.89</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00135</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-14T16:26:22.688654+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5463</v>
+      </c>
+      <c r="F4" t="n">
+        <v>39.86</v>
+      </c>
+      <c r="G4" t="n">
+        <v>72.95999999999999</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00111</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>33.1</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -580,7 +666,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -590,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-4.64</v>
+        <v>34.71</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>39.35</v>
       </c>
     </row>
     <row r="8">
@@ -620,7 +706,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>8.48</v>
       </c>
     </row>
     <row r="10">
@@ -630,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3174.169999999999</v>
+        <v>3213.519999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,183 +767,202 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>-70.34</v>
+        <v>478.57</v>
       </c>
       <c r="E15" t="n">
-        <v>-4.64</v>
+        <v>28.46</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-11.9</v>
+      </c>
+      <c r="E16" t="n">
+        <v>6.25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-70.34</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-4.64</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>118.75</v>
+      </c>
+      <c r="E18" t="n">
+        <v>28.46</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>-149.25</v>
+        <v>347.92</v>
       </c>
       <c r="E19" t="n">
-        <v>-4.64</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>78.91</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>383.29</v>
+      </c>
+      <c r="E21" t="n">
+        <v>39.35</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>78.91</v>
+        <v>146.22</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>-4.64</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-62.84</v>
+      </c>
+      <c r="E23" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="n">
-        <v>-149.25</v>
-      </c>
-      <c r="E23" t="n">
-        <v>-4.64</v>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>362.48</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>104.19</v>
+      </c>
+      <c r="E26" t="n">
+        <v>34.71</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" t="n">
-        <v>-4.64</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -879,169 +984,319 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>-4.64</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>28.46</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>6.25</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" t="n">
-        <v>-4.64</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>28.46</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" t="n">
-        <v>-4.64</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-4.64</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>-4.64</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>33.1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>39.35</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-4.64</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>33.1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.61</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>33.1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-4.64</v>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-14 22:41
</commit_message>
<xml_diff>
--- a/reports/2026-10-14.xlsx
+++ b/reports/2026-10-14.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,92 @@
       </c>
       <c r="K4" t="n">
         <v>33.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:11:32.716055+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F5" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>18</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00113</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>8.460000000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-14T20:13:10.903768+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.804</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.00134</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>8.4</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -646,7 +732,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -666,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6">
@@ -676,7 +762,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34.71</v>
+        <v>51.57</v>
       </c>
     </row>
     <row r="7">
@@ -686,7 +772,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39.35</v>
+        <v>56.21</v>
       </c>
     </row>
     <row r="8">
@@ -706,7 +792,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8.48</v>
+        <v>12.11</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +802,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3213.519999999999</v>
+        <v>3230.379999999999</v>
       </c>
     </row>
     <row r="12">
@@ -767,16 +853,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>478.57</v>
+        <v>1133.47</v>
       </c>
       <c r="E15" t="n">
-        <v>28.46</v>
+        <v>45.32</v>
       </c>
     </row>
     <row r="16">
@@ -808,494 +894,580 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>118.75</v>
+        <v>259.14</v>
       </c>
       <c r="E18" t="n">
-        <v>28.46</v>
+        <v>16.86</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>347.92</v>
+        <v>217.49</v>
       </c>
       <c r="E19" t="n">
-        <v>6.25</v>
+        <v>28.46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>644.9400000000001</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>3</v>
-      </c>
-      <c r="C21" t="n">
-        <v>3</v>
-      </c>
-      <c r="D21" t="n">
-        <v>383.29</v>
-      </c>
-      <c r="E21" t="n">
-        <v>39.35</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D22" t="n">
-        <v>146.22</v>
+        <v>822.79</v>
       </c>
       <c r="E22" t="n">
-        <v>-4.64</v>
+        <v>47.81</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>-62.84</v>
+        <v>262.88</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>6</v>
-      </c>
-      <c r="C25" t="n">
-        <v>5</v>
-      </c>
-      <c r="D25" t="n">
-        <v>362.48</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>104.19</v>
+        <v>148.31</v>
       </c>
       <c r="E26" t="n">
-        <v>34.71</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" t="n">
+        <v>609.9299999999999</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" t="n">
+        <v>363.33</v>
+      </c>
+      <c r="E28" t="n">
+        <v>51.57</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>28.46</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>6.25</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>16.86</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>28.46</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" t="n">
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>28.46</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
         <v>6.25</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>45.32</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>-4.64</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
         <v>6.25</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>33.1</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-4.64</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6.25</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>39.35</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>-4.64</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>8.460000000000001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>8.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>33.1</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B49" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>47.81</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
         <v>2</v>
       </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" t="n">
-        <v>1.61</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3.76</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" t="n">
-        <v>33.1</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>2</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="n">
+        <v>41.56</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="n">
+        <v>10.01</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" t="n">
+        <v>49.96</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
         <v>1.61</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-10-15 04:21
</commit_message>
<xml_diff>
--- a/reports/2026-10-14.xlsx
+++ b/reports/2026-10-14.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,6 +687,49 @@
       </c>
       <c r="K6" t="n">
         <v>8.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-14T23:43:35.004615+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5042</v>
+      </c>
+      <c r="F7" t="n">
+        <v>95.8</v>
+      </c>
+      <c r="G7" t="n">
+        <v>190</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00104</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>94.2</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -732,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -752,7 +795,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="6">
@@ -762,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>51.57</v>
+        <v>145.77</v>
       </c>
     </row>
     <row r="7">
@@ -772,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>56.21</v>
+        <v>150.41</v>
       </c>
     </row>
     <row r="8">
@@ -792,7 +835,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12.11</v>
+        <v>32.42</v>
       </c>
     </row>
     <row r="10">
@@ -802,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3230.379999999999</v>
+        <v>3329.479999999999</v>
       </c>
     </row>
     <row r="12">
@@ -853,16 +896,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D15" t="n">
-        <v>1133.47</v>
+        <v>1433.28</v>
       </c>
       <c r="E15" t="n">
-        <v>45.32</v>
+        <v>139.52</v>
       </c>
     </row>
     <row r="16">
@@ -898,16 +941,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>259.14</v>
+        <v>417.97</v>
       </c>
       <c r="E18" t="n">
-        <v>16.86</v>
+        <v>111.06</v>
       </c>
     </row>
     <row r="19">
@@ -917,13 +960,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>217.49</v>
+        <v>358.47</v>
       </c>
       <c r="E19" t="n">
         <v>28.46</v>
@@ -962,16 +1005,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D22" t="n">
-        <v>822.79</v>
+        <v>1122.6</v>
       </c>
       <c r="E22" t="n">
-        <v>47.81</v>
+        <v>142.01</v>
       </c>
     </row>
     <row r="23">
@@ -1045,13 +1088,13 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>9</v>
+      </c>
+      <c r="C27" t="n">
         <v>8</v>
       </c>
-      <c r="C27" t="n">
-        <v>7</v>
-      </c>
       <c r="D27" t="n">
-        <v>609.9299999999999</v>
+        <v>750.91</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1064,16 +1107,16 @@
         </is>
       </c>
       <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="n">
         <v>5</v>
       </c>
-      <c r="C28" t="n">
-        <v>4</v>
-      </c>
       <c r="D28" t="n">
-        <v>363.33</v>
+        <v>522.16</v>
       </c>
       <c r="E28" t="n">
-        <v>51.57</v>
+        <v>145.77</v>
       </c>
     </row>
     <row r="30">
@@ -1112,13 +1155,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>16.86</v>
+        <v>111.06</v>
       </c>
     </row>
     <row r="34">
@@ -1182,13 +1225,13 @@
         </is>
       </c>
       <c r="B38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" t="n">
         <v>4</v>
       </c>
-      <c r="C38" t="n">
-        <v>3</v>
-      </c>
       <c r="D38" t="n">
-        <v>45.32</v>
+        <v>139.52</v>
       </c>
     </row>
     <row r="39">
@@ -1309,166 +1352,182 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>94.2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>3</v>
-      </c>
-      <c r="C49" t="n">
-        <v>3</v>
-      </c>
-      <c r="D49" t="n">
-        <v>47.81</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="n">
+        <v>142.01</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>0.55–0.60</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B51" t="n">
         <v>2</v>
       </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
         <v>3.76</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>2</v>
-      </c>
-      <c r="C53" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" t="n">
-        <v>41.56</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>3</v>
       </c>
       <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>135.76</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
         <v>2</v>
       </c>
-      <c r="D54" t="n">
+      <c r="D55" t="n">
         <v>10.01</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>3</v>
-      </c>
-      <c r="C57" t="n">
-        <v>3</v>
-      </c>
-      <c r="D57" t="n">
-        <v>49.96</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3</v>
+      </c>
+      <c r="D58" t="n">
+        <v>49.96</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B58" t="n">
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
         <v>2</v>
       </c>
-      <c r="C58" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" t="n">
-        <v>1.61</v>
+      <c r="D59" t="n">
+        <v>95.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>